<commit_message>
Équivalences HGC/Canplast : ajout du statut Nomenclature (déjà traité)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016aozrCoPwmDDuS93STXjFo
</commit_message>
<xml_diff>
--- a/equivalences_HGC_Canplast.xlsx
+++ b/equivalences_HGC_Canplast.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Déjà liées HGC-Canplast" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 À traiter - candidat Canplast" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 HGC sans équivalent Canplast" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Déjà traitées (Nomenclature)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -31,12 +32,22 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -51,9 +62,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -497,6 +510,11 @@
           <t>Ø identique ?</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>N° INDUNI (Nomenclature) si traité</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -555,6 +573,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>381100022</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -603,10 +626,14 @@
           <t>110</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>À VÉRIFIER</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>380700001</t>
         </is>
       </c>
     </row>
@@ -667,6 +694,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>381200001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -725,6 +757,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>380300005</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -783,6 +820,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>380300006</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -841,6 +883,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>380300007</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -899,6 +946,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>380300008</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -957,6 +1009,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>380300009</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1015,6 +1072,11 @@
           <t>À VÉRIFIER</t>
         </is>
       </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>380300001</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1073,6 +1135,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>380300002</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1131,6 +1198,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>380700002</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1189,6 +1261,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>380300003</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1247,6 +1324,11 @@
           <t>À VÉRIFIER</t>
         </is>
       </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>380300004</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1305,6 +1387,11 @@
           <t>À VÉRIFIER</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>HGC et Canplast sous des n° différents</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1363,6 +1450,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>381100024</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1421,6 +1513,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>381100025</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1479,6 +1576,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>381100018</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1537,6 +1639,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>381100001</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1595,6 +1702,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>seulement Canplast</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1653,6 +1765,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>NON traité dans la nomenclature</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1711,6 +1828,11 @@
           <t>À VÉRIFIER</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>seulement Canplast</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1769,6 +1891,11 @@
           <t>À VÉRIFIER</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>HGC et Canplast sous des n° différents</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1827,6 +1954,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>381100021</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1885,6 +2017,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>381100026</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1943,6 +2080,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>381100027</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2001,6 +2143,11 @@
           <t>À VÉRIFIER</t>
         </is>
       </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>381100028</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2059,6 +2206,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>381100009</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2117,6 +2269,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>381100010</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2175,6 +2332,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>381100008</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2233,6 +2395,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>381100004</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2291,6 +2458,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>381100011</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2349,6 +2521,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>381100012</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2407,6 +2584,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>381100013</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2465,6 +2647,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>381100005</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2523,6 +2710,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>381100014</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2581,6 +2773,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>381100015</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2639,6 +2836,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>381100016</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2697,6 +2899,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>381100006</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2755,6 +2962,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>HGC et Canplast sous des n° différents</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2813,6 +3025,11 @@
           <t>OUI</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>HGC et Canplast sous des n° différents</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2869,6 +3086,11 @@
       <c r="L42" t="inlineStr">
         <is>
           <t>OUI</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>381100003</t>
         </is>
       </c>
     </row>
@@ -2883,7 +3105,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2961,6 +3183,11 @@
           <t>Critères (type, Ø, angle, longueur, SN)</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Nomenclature : Canplast déjà traité ?</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3017,6 +3244,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100009 avec autre réf HGC 100099820 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3073,6 +3305,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100011 avec autre réf HGC 100099826 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3129,6 +3366,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100014 avec autre réf HGC 100099830 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3185,6 +3427,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100010 avec autre réf HGC 100099821 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3241,6 +3488,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100012 avec autre réf HGC 100099827 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3297,6 +3549,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100015 avec autre réf HGC 100099831 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3353,6 +3610,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100008 avec autre réf HGC 100099799 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3409,6 +3671,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100013 avec autre réf HGC 100099828 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3465,6 +3732,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100016 avec autre réf HGC 100099832 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3521,6 +3793,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100004 avec autre réf HGC 100084978 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3577,6 +3854,11 @@
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100005 avec autre réf HGC 100084980 : article HGC doublon à relier ou non</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3631,6 +3913,11 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>type+Ø exact+angle+longueur (SN non comparé)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>OUI, n° INDUNI 381100006 avec autre réf HGC 100084981 : article HGC doublon à relier ou non</t>
         </is>
       </c>
     </row>
@@ -8637,4 +8924,1848 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N° INDUNI</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Désignation Induni</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Réf HGC</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Désignation HGC</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Réf Canplast</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Désignation Canplast</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Lié dans l'e-shop (equivalenceKey) ?</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ø HGC</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ø Canplast</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Remarque</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>380300001</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN2 160mm - 5m</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>100092505</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>LDT1605</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN2 Ø 160 x 3.2 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>160</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Ø différent : à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>380300002</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN2 200mm - 5m</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>100092506</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø200mm L5m</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LDT2005</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN2 Ø 200 x 3.9 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>380300003</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN2 250mm - 5m</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>100092535</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø250mm L5m</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>LDT2505</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN2 Ø 250 x 4.9 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>380300004</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN2 315mm - 5m</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>100092536</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø300mm L5m</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>LDT3155</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN2 Ø 315 x 6.2 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>315</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Ø différent : à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>380300005</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN4 125mm - 1m</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>100099739</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L1m</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LDT1251</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=1 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>380300006</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN4 125mm - 2m</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>100099800</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L2m</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LDT1252</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=2 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>380300007</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN4 125mm - 5m</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>100099801</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L5m</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LDT1255</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>380300008</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN4 200mm - 5m</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>100099806</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø200mm L5m</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>RGT2005</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN4 Ø 200 x 4,9 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>380300009</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN4 250mm - 5m</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>100099807</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø250mm L5m</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>RGT2505</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Tuyau PVC COMPACT SN4 Ø 250 x 6,2 mm L=5 M, joint incorporé</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>380700001</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau drainage flexible/Ondulé PE 110mm - 50 m</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>100037467</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Drainage flexible HDPE double paroi Ø110mm L50m</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>FLTPE110</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Tuyau de drainage HDPE double paroi Ø int./ext. 94/110 mm, rouleaux de 50 M</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Ø différent : à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>380700002</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Tuyau drainage/Perforé PVC Compact SN4 125mm - 5 m</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>100092515</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tuyau drainage PVC compact SN4 perforé a.manchon s.joint Ø125mm L5m</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LDTP125</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Tuyau de drainage PVC COMPACT, normalisé SN4 LD-TP Ø 125 mm L=5 M SANS joint</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>381100001</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Bouchon PVC 125mm à emboitement</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>100099890</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC KGM Ø125mm</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LDB125</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Bouchon PVC Ø 125 mm pour emboîtement</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>381100002</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bouchon PVC 200mm à emboitement</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>100098774</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC dur KGM Ø200mm</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LDB200</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Bouchon PVC Ø 200 mm pour emboîtement</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NON</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>381100003</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Coude PVC SN2 500 mm 90°</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>100024054</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø500mm</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LDC50090</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Coude PVC SN2 Ø 500 mm 90° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>381100004</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 125mm 90°</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>100084978</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø125mm</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LDC12590</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 125 mm 90° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>381100005</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 200mm 90°</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>100084980</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø200mm</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LDC20090</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 200 mm 90° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>381100006</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 250mm 90°</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>100084981</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø250mm</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LDC25090</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 250 mm 90° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>381100007</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Coude PVC SN2 400mm 45°</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LDC40045</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Coude PVC SN2 Ø 400 mm 45° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Canplast seul (pas d'équivalent HGC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>381100008</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 125mm 45°</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>100099799</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø125mm</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LDC12545</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 125 mm 45° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>381100009</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 125mm 15°</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>100099820</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø125mm</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LDC12515</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 125 mm 15° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>381100010</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 125mm 30°</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>100099821</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø125mm</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LDC12530</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 125 mm 30° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>381100011</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 200mm 15°</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>100099826</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø200mm</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LDC20015</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 200 mm 15° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>381100012</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 200mm 30°</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>100099827</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø200mm</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LDC20030</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 200 mm 30° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>381100013</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 200mm 45°</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>100099828</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø200mm</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LDC20045</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 200 mm 45° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>381100014</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 250mm 15°</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>100099830</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø250mm</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LDC25015</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 250 mm 15° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>381100015</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 250mm 30°</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>100099831</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø250mm</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LDC25030</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 250 mm 30° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>381100016</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 250mm 45°</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>100099832</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø250mm</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LDC25045</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Coude PVC SN4 Ø 250 mm 45° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>381100017</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Coude PVC  SN2 400mm 90°</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LDC40090</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Coude PVC SN2 Ø 400 mm 90° joint incorporé</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Canplast seul (pas d'équivalent HGC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>381100018</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embranchement PVC  SN4 250/200mm 45° </t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>100095604</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Embranchement PVC dur 45° KGEA Ø250/200mm</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LDEY250200</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Embranchement (culotte) PVC SN4 Ø 250/200 mm 45° joints incorporés</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>250/200</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>250/200</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>381100019</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embranchement PVC  SN4 110/100mm 45° </t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LDEY110110</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Embranchement (culotte) PVC SN4 Ø 110/110 mm 45° joints incorporés</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>110/110</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Canplast seul (pas d'équivalent HGC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>381100020</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embranchement PVC  SN4 125/110mm 45° </t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LDEY125110</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Embranchement (culotte) PVC SN4 Ø 125/110 mm 45° joints incorporés</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>125/110</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Canplast seul (pas d'équivalent HGC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>381100021</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embranchement PVC  SN4 125/125mm 45° </t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>100098807</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Embranchement PVC dur 45° KGEA Ø125/125mm</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LDEY125125</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Embranchement (culotte) PVC SN4 Ø 125/125 mm 45° joints incorporés</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>125/125</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>125/125</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>381100022</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 250mm</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>100023699</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Manchon double PVC dur KGMM Ø250mm</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LDDM250</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 Ø 250 mm joints incorporés</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>381100023</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 110mm</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LDDM110</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 Ø 110 mm joints incorporés</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Canplast seul (pas d'équivalent HGC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>381100024</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 125mm</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>100092563</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Manchon double PVC dur KGMM Ø125mm</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LDDM125</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 Ø 125 mm joints incorporés</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>381100025</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 200mm</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>100092565</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Manchon double PVC dur KGMM Ø200mm</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LDDM200</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Manchon double PVC SN4 Ø 200 mm joints incorporés</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>381100026</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC SN4 125mm</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>100098825</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC dur KGU Ø125mm</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LDMC125</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC SN4 Ø 125 mm joints incorporés</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>381100027</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC SN4 250mm</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>100098828</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC dur KGU Ø250mm</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LDMC250</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC SN4 Ø 250 mm joints incorporés</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>381100028</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Réduction PVC  SN4 125mm / 110mm</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>100098830</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Réduction PVC dur KGR Ø125/100mm</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>LDR125110</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Réduction PVC Ø 125/110 mm joint incorporé SN4</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>125/100</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>125/110</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Ø différent : à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>381200001</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Manchon double PEHD K55 63 mm</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>100054046</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>K 55 PEHD manchon double a. joint Ø 63mm Swisscom 1335181</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>CLPEK55MD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Manchon double pour K55 Ø63 mm</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>OUI</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Équivalences HGC/Canplast : articles HGC pas encore regardés en bleu
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016aozrCoPwmDDuS93STXjFo
</commit_message>
<xml_diff>
--- a/equivalences_HGC_Canplast.xlsx
+++ b/equivalences_HGC_Canplast.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equivalences HGC-Canplast" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Equivalences HGC-Canplast'!$A$1:$K$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Equivalences HGC-Canplast'!$A$1:$K$196</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -31,7 +31,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -66,12 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3128,8 +3134,4771 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>100001819</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>TEGUPRES 18  tuyau d'eau en caoutchouc  Ø19mm L20m</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>112.32</v>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>100001851</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>TEGUPRES 18  tuyau d'eau en caoutchouc  Ø19mm L40m</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>224.64</v>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>100001859</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bride p.tuyau d'arrosage  Ø19-28mm</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>100001963</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TEGUFIX raccord rapide filetage ext.  1"</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>100001969</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TEGUFIX raccord rapide filetage int.  3/4"</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>100002022</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TEGUFIX raccord rapide filetage int.  1"</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>100002120</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>TEGUFIX raccord type S filetage ext.  mâle Ø19mm 3/4"</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>100002180</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TEGUFIX raccord type S filetage int.  femelle Ø19mm 3/4"</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>100002187</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>TEGUFIX lance d'arrosage avec  raccord rapide 3/4"</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>100002231</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>TEGUFIX raccord rapide avec douille  Ø19mm</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>100004801</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Regard en fonte Normroll C250 Fig.2645 type 060 Mod.00</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>300.99</v>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>100004805</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Regard en fonte A15 Fig.2612 type 060 Mod.00</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>139.52</v>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>100004807</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Regard en fonte Normroll D400 Fig.2650 type 060 Mod.00</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>366.36</v>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>100004913</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Regard en fonte B125 Fig.2613 type 060 Mod.00</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>167.33</v>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>100004967</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Regard en fonte A15 Fig.2640 type 060 Mod.00 inodore</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>159.52</v>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>100004969</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Regard en fonte A15 Fig.2640 type 080 Mod.00 inodore</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>402.45</v>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>100005011</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Regard en fonte B125 Fig.2642 type 030 Mod.00 inodore</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>98.54000000000001</v>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>100005015</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Regard en fonte B125 Fig.2642 type 050 Mod.00 inodore</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>142.45</v>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>100005017</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Regard en fonte B125 Fig.2642 type 060 Mod.00 inodore</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>178.55</v>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>100005019</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Regard en fonte B125 Fig.2642 type 080 Mod.00 inodore</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>552.22</v>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>100005049</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Regard en fonte A15 Fig.2660 type 060 Mod.03 inodore</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>287.33</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>100006411</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Siphon de sol en fonte Fig.1600 type 004 Mod.00</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>91.59</v>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>100006415</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Siphon de sol en fonte Fig.1600 type 008 Mod.00</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>162.92</v>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>100006465</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Siphon de sol en fonte Fig.1601 type 010 Mod.00</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>215.95</v>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>100010087</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Clé p.regard en fonte Fig.3270 type 001 Mod.00</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>35.55</v>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>100013799</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Tuyau distanceur rugueux  26/32mm L50m</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>75.65000000000001</v>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>100013851</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Tuyau distanceur rugueux  22/26mm L50m</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>28.47</v>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>100016759</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Cadre de grille p.sac circulaire TE  Ø100/14cm</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>117.19</v>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>100/14</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>100018834</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ACO Multiline V100 S Drainlock cadre acier zinguée 0.0 L100cm</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>113.58</v>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>100018870</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>ACO Multiline V100 S Drainlock cadre acier zinguée 0.2 L50cm</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>115.49</v>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr"/>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>100019272</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ACO Multiline V100 grille passerelle A SK acier zinguée L100cm</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>50.59</v>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>100020661</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ACO Multiline V200 S Drainlock cadre acier zinguée 0.0 L100cm</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>235.75</v>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>100022532</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>ACO Multiline V100 grille fonte GGG C KTL L50cm</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>72.53</v>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>100022725</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø100mm L5m</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>100022727</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø125mm L5m</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>100022512</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø350mm L5m</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>61.84</v>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>100033022</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Tuyau de protec.câble PELD a.manch.KRSEM Ø60mm L5m</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>100033489</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Coude PELD 90° prot.câble Varioflex a.manch.90° R 600 L900mm Ø60mm</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>53.78</v>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>100033515</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Coude PELD 90° prot.câble Varioflex a.manch.90° R 1200 L1800mm Ø120mm</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>109.08</v>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>100036836</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Tuyau drainage PVC structuré SN2 perforé a.manchon s.joint Ø125mm L5m</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>5.95</v>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>100036839</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Tuyau drainage PVC structuré SN2 perforé a.manchon s.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>100040986</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Tangit colle pour tuyau PVC  500gr</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>45.08</v>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>100045336</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Scie à arc montée a.tuyau acier  L80cm</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>14.34</v>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>100046517</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Spatule coudée de plâtrier inoxidable  60mm</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>100046519</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Spatule coudée de plâtrier inoxidable  70mm</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>100046561</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Spatule coudée de plâtrier inoxidable  80mm</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>100046657</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>MSU échelon en aluminium coudé 350</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>26.33</v>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>100051224</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Grille de ventilation alu manchonnée Ø300mm avec treillis moustiquaire</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>73.63</v>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>100053897</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>KW 50 PEHD tuyau ondulé, int.lisse Ø 63mm L 100m Swisscom 1337666</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>100053899</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>K 55 HDPE tuyau manch. blanc/gris Ø 63mm L 5m Swisscom 1337435</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>100053921</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>K 55 HDPE tuyau manch. blanc/gris Ø 63mm L 10m Swisscom 1337427</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>100053925</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>K100 PELD tuyau prot. câble a. fermet-L Ø 112mm L 10m Swisscom 1338284</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>32.12</v>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>100053927</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>K120 PELD tuyau prot.câble a. fermet-L Ø 132mm L 10m Swisscom 1338888</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>100053954</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>K 55 PEDH coude 90° Ø63mm R0.6m L1.6m Swisscom 1337567</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>17.55</v>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>100053980</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>K100 PE manchon double a. fermeture-L Ø 112mm Swisscom 1338292</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>30.17</v>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>100054011</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>K 55 PEHD manchon rétractable 63/55/260mm Swisscom 1335157</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>16.59</v>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>100054103</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Raccord pour canal câble 4  incl. set montage Swisscom 1337732</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>174</v>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>100054289</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Tuyau d'acier droit 60.3x2.9mm  L 700mm Swisscom 1302413</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>33</v>
+      </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>100054343</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Caniveau de câbles no.4 80/110/43mm zingué 2pc. à L 6m Swisscom 1300441</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>160</v>
+      </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>100054348</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Bride p. caniveau de câbles no.4 deux pièces zinguées Swisscom 1300839</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>100054418</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Enkadrain natte de drainage CKL 20 20mm 100cm L30m</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>801.99</v>
+      </c>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>100054464</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Delta-Terraxx natte de drainage 240cm L12.5m</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>304.96</v>
+      </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>100059031</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Tuyau pour  zu Spray-Matic 10B  incl. connections</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>100062871</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Delta-Terraxx R natte de drainage 240cm L12.5m</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>268.94</v>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>100099736</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø100mm L1m</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>100099737</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø100mm L2m</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>100099738</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø100mm L5m</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>100099802</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø150mm L1m</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>100099284</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø150mm L2m</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>100099803</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>100099804</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø200mm L1m</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>16.91</v>
+      </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>100099805</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø200mm L2m</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>15.39</v>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>100099808</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø300mm L5m</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>41.12</v>
+      </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>100068660</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Lance p.tuyau d'arrosage Stop Net</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>129</v>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>100081659</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>ACO Multiline V200 grille fonte D/E600 SK Design revêtement KTL L50cm</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>195.66</v>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>100084436</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Tuyau de protec.câble HDPE a.manch.blanc Ø120mm L5m</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>5.84</v>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>100092516</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Tuyau drainage PVC compact SN4 perforé a.manchon s.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>11.564</v>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>100092564</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Manchon double PVC dur KGMM Ø150mm</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>100099889</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC KGM Ø100mm</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>100099891</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC KGM Ø150mm</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>100099894</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC KGM Ø300mm</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>33.66</v>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>100098799</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 87° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>100098804</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 87° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>56.33</v>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>100098809</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Embranchement PVC dur 45° KGEA Ø150/125mm</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>150/125</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr"/>
+      <c r="J139" t="inlineStr"/>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>100098810</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Embranchement PVC dur 45° KGEA Ø150/150mm</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>150/150</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr"/>
+      <c r="J140" t="inlineStr"/>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>100098813</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Embranchement PVC dur 45° KGEA Ø200/150mm</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>18.13</v>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>200/150</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>100098824</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC dur KGU Ø100mm</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr"/>
+      <c r="G142" t="inlineStr"/>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr"/>
+      <c r="J142" t="inlineStr"/>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>100098826</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Manchon coulissant PVC dur KGU Ø150mm</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr"/>
+      <c r="J143" t="inlineStr"/>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>100098832</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Réduction PVC dur KGR Ø150/125mm</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
+      <c r="G144" t="inlineStr"/>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>150/125</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>100098834</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Réduction PVC dur KGR Ø200/150mm</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>200/150</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>100098859</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Manchon double PEHD p.tuyau câble KRDM Ø120mm</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>7.92</v>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr"/>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>100098992</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Tuyau de protec.câble LDPE a.manch.blanc C+S Ø60mm L5m</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>100098995</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Tuyau de protec.câble LDPE a.manch.blanc C+S Ø120mm L5m</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr"/>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>100053989</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>K120 PEHD manchon de réparation Ø 132mm a. ferm. longitudinale Swisscom 1338912</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>37.45</v>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr"/>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr"/>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>100056934</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>K120 PEHD manchon de réparation Ø 132mm Swisscom 1338904</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>6.99</v>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>132</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr"/>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>100099794</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr"/>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>100099822</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>100099833</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>48.16</v>
+      </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>100099795</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr"/>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>100099823</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr"/>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>100099834</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>49.34</v>
+      </c>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr"/>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>100099796</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr"/>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>100099824</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr"/>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>100099835</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>54.55</v>
+      </c>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr"/>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>100084977</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr"/>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>100084979</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr"/>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr"/>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>100084982</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>110.37</v>
+      </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr"/>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>100095519</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr"/>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>100095571</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr"/>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>100095574</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>100024056</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 15° KGB incl.joint Ø350mm</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>152.44</v>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr"/>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>100095575</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr"/>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr"/>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>100095577</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr"/>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>100095580</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr"/>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>100023481</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 30° KGB incl.joint Ø350mm</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>171.04</v>
+      </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr"/>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr"/>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>100095581</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr"/>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr"/>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>100095583</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I172" t="inlineStr"/>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>100095586</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>64.95999999999999</v>
+      </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr"/>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>100023570</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 45° KGB incl.joint Ø350mm</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>196.32</v>
+      </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>100095592</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø100mm</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr"/>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>100095594</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø150mm</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>100095597</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø300mm</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>70.12</v>
+      </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>100023667</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø350mm</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>270.69</v>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>100063110</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr"/>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>100063111</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø200mm L5m</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>16.42</v>
+      </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>100063112</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø250mm L5m</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>27.14</v>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr"/>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>100063113</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø300mm L5m</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>44.07</v>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr"/>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>100124017</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN2 structuré a.manchon a.joint Ø400mm L5m</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>74.86</v>
+      </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>100063068</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø100mm L5m</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>6.35</v>
+      </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>100063069</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø125mm L5m</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>8.41</v>
+      </c>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>100072421</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr"/>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>100072422</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø200mm L5m</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>19.82</v>
+      </c>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr"/>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr"/>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>100072423</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø250mm L5m</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>33.23</v>
+      </c>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr"/>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>100072424</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø300mm L5m</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>52.61</v>
+      </c>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr"/>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr"/>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>100124018</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN4 structuré a.manchon a.joint Ø400mm L5m</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>90.98</v>
+      </c>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="inlineStr"/>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>100073688</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN8 structuré a.manchon a.joint Ø100mm L5m</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>6.73</v>
+      </c>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr"/>
+      <c r="J191" t="inlineStr"/>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>100073689</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN8 structuré a.manchon a.joint Ø125mm L5m</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>9.050000000000001</v>
+      </c>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>100067724</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN8 structuré a.manchon a.joint Ø150mm L5m</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>11.11</v>
+      </c>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr"/>
+      <c r="J193" t="inlineStr"/>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>100067725</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN8 structuré a.manchon a.joint Ø200mm L5m</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>22.97</v>
+      </c>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr"/>
+      <c r="J194" t="inlineStr"/>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>100067726</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN8 structuré a.manchon a.joint Ø250mm L5m</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>37.78</v>
+      </c>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr"/>
+      <c r="J195" t="inlineStr"/>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="5" t="inlineStr">
+        <is>
+          <t>Pas encore regardé</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>100124019</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Tuyau PVC SN8 structuré a.manchon a.joint Ø400mm L5m</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>98.23</v>
+      </c>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr"/>
+      <c r="J196" t="inlineStr"/>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Aucun Canplast de même Ø exact trouvé automatiquement : à vérifier à la main</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K55"/>
+  <autoFilter ref="A1:K196"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Équivalences HGC/Canplast : n° INDUNI repris aussi côté Canplast
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016aozrCoPwmDDuS93STXjFo
</commit_message>
<xml_diff>
--- a/equivalences_HGC_Canplast.xlsx
+++ b/equivalences_HGC_Canplast.xlsx
@@ -1454,15 +1454,15 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Embranchement 45° PVC (Y)</t>
+          <t>Coudes PVC</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>381100018</v>
+        <v>381100007</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Embranchement PVC  SN4 250/200mm 45° </t>
+          <t>Coude PVC SN2 400mm 45°</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1472,38 +1472,38 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>100095604</t>
+          <t>100095587</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Embranchement PVC dur 45° KGEA Ø250/200mm</t>
+          <t>Coude PVC dur 45° KGB incl.joint Ø400mm</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>59.6</v>
+        <v>162.37</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>LDEY250200</t>
+          <t>LDC40045</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Embranchement (culotte) PVC SN4 Ø 250/200 mm 45° joints incorporés</t>
+          <t>Coude PVC SN2 Ø 400 mm 45° joint incorporé</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>37.77</v>
+        <v>103.41</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>250/200</t>
+          <t>400</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>250/200</t>
+          <t>400</t>
         </is>
       </c>
     </row>
@@ -1537,11 +1537,11 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>381100021</v>
+        <v>381100018</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Embranchement PVC  SN4 125/125mm 45° </t>
+          <t xml:space="preserve">Embranchement PVC  SN4 250/200mm 45° </t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1551,38 +1551,38 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>100098807</t>
+          <t>100095604</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Embranchement PVC dur 45° KGEA Ø125/125mm</t>
+          <t>Embranchement PVC dur 45° KGEA Ø250/200mm</t>
         </is>
       </c>
       <c r="L14" t="n">
-        <v>6.6</v>
+        <v>59.6</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>LDEY125125</t>
+          <t>LDEY250200</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Embranchement (culotte) PVC SN4 Ø 125/125 mm 45° joints incorporés</t>
+          <t>Embranchement (culotte) PVC SN4 Ø 250/200 mm 45° joints incorporés</t>
         </is>
       </c>
       <c r="O14" t="n">
-        <v>3.93</v>
+        <v>37.77</v>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>125/125</t>
+          <t>250/200</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>125/125</t>
+          <t>250/200</t>
         </is>
       </c>
     </row>
@@ -1612,15 +1612,15 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC</t>
+          <t>Embranchement 45° PVC (Y)</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>381100026</v>
+        <v>381100021</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC SN4 125mm</t>
+          <t xml:space="preserve">Embranchement PVC  SN4 125/125mm 45° </t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1630,38 +1630,38 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>100098825</t>
+          <t>100098807</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC dur KGU Ø125mm</t>
+          <t>Embranchement PVC dur 45° KGEA Ø125/125mm</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>2.83</v>
+        <v>6.6</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>LDMC125</t>
+          <t>LDEY125125</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC SN4 Ø 125 mm joints incorporés</t>
+          <t>Embranchement (culotte) PVC SN4 Ø 125/125 mm 45° joints incorporés</t>
         </is>
       </c>
       <c r="O15" t="n">
-        <v>2.13</v>
+        <v>3.93</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>125/125</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>125/125</t>
         </is>
       </c>
     </row>
@@ -1695,11 +1695,11 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>381100027</v>
+        <v>381100026</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC SN4 250mm</t>
+          <t>Manchon coulissant PVC SN4 125mm</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1709,38 +1709,38 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>100098828</t>
+          <t>100098825</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC dur KGU Ø250mm</t>
+          <t>Manchon coulissant PVC dur KGU Ø125mm</t>
         </is>
       </c>
       <c r="L16" t="n">
-        <v>16.8</v>
+        <v>2.83</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>LDMC250</t>
+          <t>LDMC125</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Manchon coulissant PVC SN4 Ø 250 mm joints incorporés</t>
+          <t>Manchon coulissant PVC SN4 Ø 125 mm joints incorporés</t>
         </is>
       </c>
       <c r="O16" t="n">
-        <v>18.26</v>
+        <v>2.13</v>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>125</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -1765,20 +1765,20 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Canalisation</t>
+          <t>Pièces Canalisation PVC</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Canalisation PVC CR4 Compact</t>
+          <t>Manchon coulissant PVC</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>380300005</v>
+        <v>381100027</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN4 125mm - 1m</t>
+          <t>Manchon coulissant PVC SN4 250mm</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1788,38 +1788,38 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>100099739</t>
+          <t>100098828</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L1m</t>
+          <t>Manchon coulissant PVC dur KGU Ø250mm</t>
         </is>
       </c>
       <c r="L17" t="n">
-        <v>7.97</v>
+        <v>16.8</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>LDT1251</t>
+          <t>LDMC250</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=1 M, joint incorporé</t>
+          <t>Manchon coulissant PVC SN4 Ø 250 mm joints incorporés</t>
         </is>
       </c>
       <c r="O17" t="n">
-        <v>10.95</v>
+        <v>18.26</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>250</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>250</t>
         </is>
       </c>
     </row>
@@ -1844,20 +1844,20 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pièces Canalisation PVC</t>
+          <t>Canalisation</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Coudes PVC</t>
+          <t>Canalisation PVC CR4 Compact</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>381100008</v>
+        <v>380300005</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 125mm 45°</t>
+          <t>Tuyau PVC Compact SN4 125mm - 1m</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1867,29 +1867,29 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>100099799</t>
+          <t>100099739</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Coude PVC dur 45° KGB incl.joint Ø125mm</t>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L1m</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>3.25</v>
+        <v>7.97</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>LDC12545</t>
+          <t>LDT1251</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 125 mm 45° joint incorporé</t>
+          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=1 M, joint incorporé</t>
         </is>
       </c>
       <c r="O18" t="n">
-        <v>2.2</v>
+        <v>10.95</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
@@ -1923,20 +1923,20 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Canalisation</t>
+          <t>Pièces Canalisation PVC</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Canalisation PVC CR4 Compact</t>
+          <t>Coudes PVC</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>380300006</v>
+        <v>381100008</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN4 125mm - 2m</t>
+          <t>Coude PVC SN4 125mm 45°</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1946,29 +1946,29 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>100099800</t>
+          <t>100099799</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L2m</t>
+          <t>Coude PVC dur 45° KGB incl.joint Ø125mm</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>6.97</v>
+        <v>3.25</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>LDT1252</t>
+          <t>LDC12545</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=2 M, joint incorporé</t>
+          <t>Coude PVC SN4 Ø 125 mm 45° joint incorporé</t>
         </is>
       </c>
       <c r="O19" t="n">
-        <v>9.039999999999999</v>
+        <v>2.2</v>
       </c>
       <c r="P19" t="inlineStr">
         <is>
@@ -2011,11 +2011,11 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>380300007</v>
+        <v>380300006</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN4 125mm - 5m</t>
+          <t>Tuyau PVC Compact SN4 125mm - 2m</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -2025,29 +2025,29 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>100099801</t>
+          <t>100099800</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L5m</t>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L2m</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>6.3</v>
+        <v>6.97</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>LDT1255</t>
+          <t>LDT1252</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=5 M, joint incorporé</t>
+          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=2 M, joint incorporé</t>
         </is>
       </c>
       <c r="O20" t="n">
-        <v>5.83</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="P20" t="inlineStr">
         <is>
@@ -2090,11 +2090,11 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>380300008</v>
+        <v>380300007</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN4 200mm - 5m</t>
+          <t>Tuyau PVC Compact SN4 125mm - 5m</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -2104,38 +2104,38 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>100099806</t>
+          <t>100099801</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Tuyau canal.PVC SN4 incl.joint Ø200mm L5m</t>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø125mm L5m</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>14.59</v>
+        <v>6.3</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>RGT2005</t>
+          <t>LDT1255</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN4 Ø 200 x 4,9 mm L=5 M, joint incorporé</t>
+          <t>Tuyau PVC COMPACT SN4 Ø 125 x 3.2 mm L=5 M, joint incorporé</t>
         </is>
       </c>
       <c r="O21" t="n">
-        <v>13.76</v>
+        <v>5.83</v>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>125</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -2169,11 +2169,11 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>380300009</v>
+        <v>380300008</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN4 250mm - 5m</t>
+          <t>Tuyau PVC Compact SN4 200mm - 5m</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -2183,38 +2183,38 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>100099807</t>
+          <t>100099806</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Tuyau canal.PVC SN4 incl.joint Ø250mm L5m</t>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø200mm L5m</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>25.21</v>
+        <v>14.59</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>RGT2505</t>
+          <t>RGT2005</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN4 Ø 250 x 6,2 mm L=5 M, joint incorporé</t>
+          <t>Tuyau PVC COMPACT SN4 Ø 200 x 4,9 mm L=5 M, joint incorporé</t>
         </is>
       </c>
       <c r="O22" t="n">
-        <v>23.06</v>
+        <v>13.76</v>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>200</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -2239,20 +2239,20 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Pièces Canalisation PVC</t>
+          <t>Canalisation</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Coudes PVC</t>
+          <t>Canalisation PVC CR4 Compact</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>381100009</v>
+        <v>380300009</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 125mm 15°</t>
+          <t>Tuyau PVC Compact SN4 250mm - 5m</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2262,38 +2262,38 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>100099820</t>
+          <t>100099807</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Coude PVC dur 15° KGB incl.joint Ø125mm</t>
+          <t>Tuyau canal.PVC SN4 incl.joint Ø250mm L5m</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>2.95</v>
+        <v>25.21</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>LDC12515</t>
+          <t>RGT2505</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 125 mm 15° joint incorporé</t>
+          <t>Tuyau PVC COMPACT SN4 Ø 250 x 6,2 mm L=5 M, joint incorporé</t>
         </is>
       </c>
       <c r="O23" t="n">
-        <v>2.2</v>
+        <v>23.06</v>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>250</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>250</t>
         </is>
       </c>
     </row>
@@ -2327,11 +2327,11 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>381100010</v>
+        <v>381100009</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 125mm 30°</t>
+          <t>Coude PVC SN4 125mm 15°</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2341,25 +2341,25 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>100099821</t>
+          <t>100099820</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Coude PVC dur 30° KGB incl.joint Ø125mm</t>
+          <t>Coude PVC dur 15° KGB incl.joint Ø125mm</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>2.67</v>
+        <v>2.95</v>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>LDC12530</t>
+          <t>LDC12515</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 125 mm 30° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 125 mm 15° joint incorporé</t>
         </is>
       </c>
       <c r="O24" t="n">
@@ -2406,11 +2406,11 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>381100011</v>
+        <v>381100010</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 200mm 15°</t>
+          <t>Coude PVC SN4 125mm 30°</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2420,38 +2420,38 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>100099826</t>
+          <t>100099821</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Coude PVC dur 15° KGB incl.joint Ø200mm</t>
+          <t>Coude PVC dur 30° KGB incl.joint Ø125mm</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>9.41</v>
+        <v>2.67</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>LDC20015</t>
+          <t>LDC12530</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 200 mm 15° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 125 mm 30° joint incorporé</t>
         </is>
       </c>
       <c r="O25" t="n">
-        <v>7.03</v>
+        <v>2.2</v>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>125</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>125</t>
         </is>
       </c>
     </row>
@@ -2485,11 +2485,11 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>381100012</v>
+        <v>381100011</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 200mm 30°</t>
+          <t>Coude PVC SN4 200mm 15°</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -2499,25 +2499,25 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>100099827</t>
+          <t>100099826</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Coude PVC dur 30° KGB incl.joint Ø200mm</t>
+          <t>Coude PVC dur 15° KGB incl.joint Ø200mm</t>
         </is>
       </c>
       <c r="L26" t="n">
-        <v>9.75</v>
+        <v>9.41</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>LDC20030</t>
+          <t>LDC20015</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 200 mm 30° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 200 mm 15° joint incorporé</t>
         </is>
       </c>
       <c r="O26" t="n">
@@ -2564,11 +2564,11 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>381100013</v>
+        <v>381100012</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 200mm 45°</t>
+          <t>Coude PVC SN4 200mm 30°</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2578,25 +2578,25 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>100099828</t>
+          <t>100099827</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Coude PVC dur 45° KGB incl.joint Ø200mm</t>
+          <t>Coude PVC dur 30° KGB incl.joint Ø200mm</t>
         </is>
       </c>
       <c r="L27" t="n">
-        <v>10.44</v>
+        <v>9.75</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>LDC20045</t>
+          <t>LDC20030</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 200 mm 45° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 200 mm 30° joint incorporé</t>
         </is>
       </c>
       <c r="O27" t="n">
@@ -2643,11 +2643,11 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>381100014</v>
+        <v>381100013</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 250mm 15°</t>
+          <t>Coude PVC SN4 200mm 45°</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2657,38 +2657,38 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>100099830</t>
+          <t>100099828</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Coude PVC dur 15° KGB incl.joint Ø250mm</t>
+          <t>Coude PVC dur 45° KGB incl.joint Ø200mm</t>
         </is>
       </c>
       <c r="L28" t="n">
-        <v>38.3</v>
+        <v>10.44</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>LDC25015</t>
+          <t>LDC20045</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 250 mm 15° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 200 mm 45° joint incorporé</t>
         </is>
       </c>
       <c r="O28" t="n">
-        <v>23.06</v>
+        <v>7.03</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>200</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>200</t>
         </is>
       </c>
     </row>
@@ -2722,11 +2722,11 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>381100015</v>
+        <v>381100014</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 250mm 30°</t>
+          <t>Coude PVC SN4 250mm 15°</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2736,25 +2736,25 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>100099831</t>
+          <t>100099830</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Coude PVC dur 30° KGB incl.joint Ø250mm</t>
+          <t>Coude PVC dur 15° KGB incl.joint Ø250mm</t>
         </is>
       </c>
       <c r="L29" t="n">
-        <v>39.47</v>
+        <v>38.3</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>LDC25030</t>
+          <t>LDC25015</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 250 mm 30° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 250 mm 15° joint incorporé</t>
         </is>
       </c>
       <c r="O29" t="n">
@@ -2801,11 +2801,11 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>381100016</v>
+        <v>381100015</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 250mm 45°</t>
+          <t>Coude PVC SN4 250mm 30°</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2815,25 +2815,25 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>100099832</t>
+          <t>100099831</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Coude PVC dur 45° KGB incl.joint Ø250mm</t>
+          <t>Coude PVC dur 30° KGB incl.joint Ø250mm</t>
         </is>
       </c>
       <c r="L30" t="n">
-        <v>41.78</v>
+        <v>39.47</v>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>LDC25045</t>
+          <t>LDC25030</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Coude PVC SN4 Ø 250 mm 45° joint incorporé</t>
+          <t>Coude PVC SN4 Ø 250 mm 30° joint incorporé</t>
         </is>
       </c>
       <c r="O30" t="n">
@@ -2876,15 +2876,15 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Bouchon PVC</t>
+          <t>Coudes PVC</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>381100001</v>
+        <v>381100016</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Bouchon PVC 125mm à emboitement</t>
+          <t>Coude PVC SN4 250mm 45°</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2894,38 +2894,38 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>100099890</t>
+          <t>100099832</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Bouchon p.manchon PVC KGM Ø125mm</t>
+          <t>Coude PVC dur 45° KGB incl.joint Ø250mm</t>
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1.68</v>
+        <v>41.78</v>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>LDB125</t>
+          <t>LDC25045</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Bouchon PVC Ø 125 mm pour emboîtement</t>
+          <t>Coude PVC SN4 Ø 250 mm 45° joint incorporé</t>
         </is>
       </c>
       <c r="O31" t="n">
-        <v>1.11</v>
+        <v>23.06</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>250</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>250</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,11 @@
           <t>X</t>
         </is>
       </c>
-      <c r="B32" s="7" t="n"/>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="C32" t="n">
         <v>38000</v>
       </c>
@@ -2955,221 +2959,292 @@
         </is>
       </c>
       <c r="G32" t="n">
+        <v>381100001</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Bouchon PVC 125mm à emboitement</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>100099890</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC KGM Ø125mm</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>LDB125</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Bouchon PVC Ø 125 mm pour emboîtement</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>PRODUITS DE GENIE-CIVIL</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Pièces Canalisation PVC</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Bouchon PVC</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
         <v>381100002</v>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>Bouchon PVC 200mm à emboitement</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Déjà traité</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>100099892</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Bouchon p.manchon PVC KGM Ø200mm</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>LDB200</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Bouchon PVC Ø 200 mm pour emboîtement</t>
+        </is>
+      </c>
+      <c r="O33" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>PRODUITS DE GENIE-CIVIL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Pièces Canalisation PVC</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Coudes PVC</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>381100017</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Coude PVC  SN2 400mm 90°</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>100101860</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Coude PVC dur 90° KGB incl.joint Ø400mm</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>248.49</v>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>LDC40090</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Coude PVC SN2 Ø 400 mm 90° joint incorporé</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>158.25</v>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>PRODUITS DE GENIE-CIVIL</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Pièces Canalisation PVC</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Bouchon PVC</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>381100002</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Bouchon PVC 200mm à emboitement</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Déjà traité</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>100098774</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Bouchon p.manchon PVC dur KGM Ø200mm</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>absent du catalogue</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>LDB200</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>Bouchon PVC Ø 200 mm pour emboîtement</t>
         </is>
       </c>
-      <c r="O32" t="n">
+      <c r="O35" t="n">
         <v>2.63</v>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="R35" t="inlineStr">
         <is>
           <t>Dans la Nomenclature mais pas encore lié dans l'e-shop</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="n"/>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Déjà traité</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>100095587</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Coude PVC dur 45° KGB incl.joint Ø400mm</t>
-        </is>
-      </c>
-      <c r="L33" t="n">
-        <v>162.37</v>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>LDC40045</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Coude PVC SN2 Ø 400 mm 45° joint incorporé</t>
-        </is>
-      </c>
-      <c r="O33" t="n">
-        <v>103.41</v>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Lié dans l'e-shop, absent de la Nomenclature</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Déjà traité</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>100099892</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Bouchon p.manchon PVC KGM Ø200mm</t>
-        </is>
-      </c>
-      <c r="L34" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>LDB200</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Bouchon PVC Ø 200 mm pour emboîtement</t>
-        </is>
-      </c>
-      <c r="O34" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Lié dans l'e-shop, absent de la Nomenclature</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>Déjà traité</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>100099893</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Bouchon p.manchon PVC KGM Ø250mm</t>
-        </is>
-      </c>
-      <c r="L35" t="n">
-        <v>22.04</v>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>LDB250</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Bouchon PVC Ø 250 mm pour emboîtement</t>
-        </is>
-      </c>
-      <c r="O35" t="n">
-        <v>12.86</v>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>250</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Lié dans l'e-shop, absent de la Nomenclature</t>
         </is>
       </c>
     </row>
@@ -3187,38 +3262,38 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>100101860</t>
+          <t>100099893</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Coude PVC dur 90° KGB incl.joint Ø400mm</t>
+          <t>Bouchon p.manchon PVC KGM Ø250mm</t>
         </is>
       </c>
       <c r="L36" t="n">
-        <v>248.49</v>
+        <v>22.04</v>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>LDC40090</t>
+          <t>LDB250</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Coude PVC SN2 Ø 400 mm 90° joint incorporé</t>
+          <t>Bouchon PVC Ø 250 mm pour emboîtement</t>
         </is>
       </c>
       <c r="O36" t="n">
-        <v>158.25</v>
+        <v>12.86</v>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>250</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>250</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3228,12 +3303,42 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="7" t="n"/>
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
+      <c r="C37" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>PRODUITS DE GENIE-CIVIL</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Drainage</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Tuyau Drainage PE</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>380700001</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Tuyau drainage flexible/Ondulé PE 110mm - 50 m</t>
+        </is>
+      </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
           <t>Ø différent - à confirmer</t>
@@ -3241,53 +3346,78 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>100092562</t>
+          <t>100037467</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Manchon double PVC dur KGMM Ø100mm</t>
+          <t>Drainage flexible HDPE double paroi Ø110mm L50m</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>2.41</v>
+        <v>5.34</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>LDDM110</t>
+          <t>FLTPE110</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Manchon double PVC SN4 Ø 110 mm joints incorporés</t>
+          <t>Tuyau de drainage HDPE double paroi Ø int./ext. 94/110 mm, rouleaux de 50 M</t>
         </is>
       </c>
       <c r="O37" t="n">
-        <v>1.54</v>
+        <v>3.42</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
           <t>110</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Ø différents (nominal vs réel ?)</t>
+          <t>Ø différents (nominal vs réel ?) (dans la Nomenclature)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="n"/>
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
+      <c r="C38" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>PRODUITS DE GENIE-CIVIL</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Canalisation</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Canalisation PVC CR2 Compact</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>380300001</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN2 160mm - 5m</t>
+        </is>
+      </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
           <t>Ø différent - à confirmer</t>
@@ -3295,53 +3425,83 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>100098805</t>
+          <t>100092505</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Embranchement PVC dur 45° KGEA Ø100/100mm</t>
+          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø150mm L5m</t>
         </is>
       </c>
       <c r="L38" t="n">
-        <v>4.93</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>LDEY110110</t>
+          <t>LDT1605</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Embranchement (culotte) PVC SN4 Ø 110/110 mm 45° joints incorporés</t>
+          <t>Tuyau PVC COMPACT SN2 Ø 160 x 3.2 mm L=5 M, joint incorporé</t>
         </is>
       </c>
       <c r="O38" t="n">
-        <v>2.89</v>
+        <v>7.48</v>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>100/100</t>
+          <t>150</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>110/110</t>
+          <t>160</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Ø différents (nominal vs réel ?)</t>
+          <t>Ø différents (nominal vs réel ?) (dans la Nomenclature)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="n"/>
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
+      <c r="C39" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>PRODUITS DE GENIE-CIVIL</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Canalisation</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Canalisation PVC CR2 Compact</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>380300004</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Tuyau PVC Compact SN2 315mm - 5m</t>
+        </is>
+      </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
           <t>Ø différent - à confirmer</t>
@@ -3349,43 +3509,43 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>100098806</t>
+          <t>100092536</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Embranchement PVC dur 45° KGEA Ø125/100mm</t>
+          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø300mm L5m</t>
         </is>
       </c>
       <c r="L39" t="n">
-        <v>5.56</v>
+        <v>34.106</v>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>LDEY125110</t>
+          <t>LDT3155</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Embranchement (culotte) PVC SN4 Ø 125/110 mm 45° joints incorporés</t>
+          <t>Tuyau PVC COMPACT SN2 Ø 315 x 6.2 mm L=5 M, joint incorporé</t>
         </is>
       </c>
       <c r="O39" t="n">
-        <v>3.93</v>
+        <v>30.59</v>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>125/100</t>
+          <t>300</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>125/110</t>
+          <t>315</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Ø différents (nominal vs réel ?)</t>
+          <t>Ø différents (nominal vs réel ?) (dans la Nomenclature)</t>
         </is>
       </c>
     </row>
@@ -3410,20 +3570,20 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Drainage</t>
+          <t>Pièces Canalisation PVC</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Tuyau Drainage PE</t>
+          <t>Manchon double PVC</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>380700001</v>
+        <v>381100023</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Tuyau drainage flexible/Ondulé PE 110mm - 50 m</t>
+          <t>Manchon double PVC SN4 110mm</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -3433,31 +3593,36 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>100037467</t>
+          <t>100092562</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Drainage flexible HDPE double paroi Ø110mm L50m</t>
+          <t>Manchon double PVC dur KGMM Ø100mm</t>
         </is>
       </c>
       <c r="L40" t="n">
-        <v>5.34</v>
+        <v>2.41</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>FLTPE110</t>
+          <t>LDDM110</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Tuyau de drainage HDPE double paroi Ø int./ext. 94/110 mm, rouleaux de 50 M</t>
+          <t>Manchon double PVC SN4 Ø 110 mm joints incorporés</t>
         </is>
       </c>
       <c r="O40" t="n">
-        <v>3.42</v>
+        <v>1.54</v>
       </c>
       <c r="P40" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
         <is>
           <t>110</t>
         </is>
@@ -3489,20 +3654,20 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Canalisation</t>
+          <t>Pièces Canalisation PVC</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Canalisation PVC CR2 Compact</t>
+          <t>Embranchement 45° PVC (Y)</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>380300001</v>
+        <v>381100019</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN2 160mm - 5m</t>
+          <t xml:space="preserve">Embranchement PVC  SN4 110/100mm 45° </t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -3512,38 +3677,38 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>100092505</t>
+          <t>100098805</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø150mm L5m</t>
+          <t>Embranchement PVC dur 45° KGEA Ø100/100mm</t>
         </is>
       </c>
       <c r="L41" t="n">
-        <v>8.869999999999999</v>
+        <v>4.93</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>LDT1605</t>
+          <t>LDEY110110</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN2 Ø 160 x 3.2 mm L=5 M, joint incorporé</t>
+          <t>Embranchement (culotte) PVC SN4 Ø 110/110 mm 45° joints incorporés</t>
         </is>
       </c>
       <c r="O41" t="n">
-        <v>7.48</v>
+        <v>2.89</v>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>100/100</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>110/110</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3573,20 +3738,20 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Canalisation</t>
+          <t>Pièces Canalisation PVC</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Canalisation PVC CR2 Compact</t>
+          <t>Embranchement 45° PVC (Y)</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>380300004</v>
+        <v>381100020</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Tuyau PVC Compact SN2 315mm - 5m</t>
+          <t xml:space="preserve">Embranchement PVC  SN4 125/110mm 45° </t>
         </is>
       </c>
       <c r="I42" s="3" t="inlineStr">
@@ -3596,38 +3761,38 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>100092536</t>
+          <t>100098806</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Tuyau PVC SN2 compact a.manchon a.joint Ø300mm L5m</t>
+          <t>Embranchement PVC dur 45° KGEA Ø125/100mm</t>
         </is>
       </c>
       <c r="L42" t="n">
-        <v>34.106</v>
+        <v>5.56</v>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>LDT3155</t>
+          <t>LDEY125110</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Tuyau PVC COMPACT SN2 Ø 315 x 6.2 mm L=5 M, joint incorporé</t>
+          <t>Embranchement (culotte) PVC SN4 Ø 125/110 mm 45° joints incorporés</t>
         </is>
       </c>
       <c r="O42" t="n">
-        <v>30.59</v>
+        <v>3.93</v>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>300</t>
+          <t>125/100</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>315</t>
+          <t>125/110</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">

</xml_diff>